<commit_message>
solomon heuristic is added
</commit_message>
<xml_diff>
--- a/inputs/config.xlsx
+++ b/inputs/config.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C53"/>
+  <dimension ref="A1:C67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -560,7 +560,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Demo supports two modes: 'single_objective' (one MIP solve) or 'multi_objective' (epsilon-constraint sweep over the Pareto front).</t>
+          <t>Three modes: 'single_objective' (one MIP solve), 'multi_objective' (epsilon-constraint Pareto sweep), or 'heuristic' (Solomon I1 only — no MIP).</t>
         </is>
       </c>
     </row>
@@ -1090,7 +1090,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t># VERIFICATION &amp; VISUALIZATION</t>
+          <t># SOLOMON I1 HEURISTIC</t>
         </is>
       </c>
       <c r="C46" s="3" t="n"/>
@@ -1098,102 +1098,307 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>auto_verify</t>
-        </is>
-      </c>
-      <c r="B47" t="b">
-        <v>1</v>
+          <t>heuristic_objective</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>route_duration</t>
+        </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>Run verify.py on the solution.</t>
+          <t>Bias label: 'route_duration' or 'wait_time'. Auto-flips the default alpha-triple.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>verify_on_fail</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>raise</t>
-        </is>
+          <t>alpha_1</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>0.0001</v>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>'raise' or 'warn' on verification failures.</t>
+          <t>Weight on Δ-distance in Solomon c_1.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>auto_visualize</t>
-        </is>
-      </c>
-      <c r="B49" t="b">
+          <t>alpha_2</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
         <v>1</v>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Render Gantt / route / wait plots after each solve.</t>
+          <t>Weight on Δ-fleet-route-duration in c_1.</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t># OUTPUT</t>
-        </is>
-      </c>
-      <c r="C50" s="3" t="n"/>
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>alpha_3</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>Weight on Δ-fleet-total-wait in c_1.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>output_dir</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>results</t>
-        </is>
+          <t>lambda_c2</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>1</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>Destination folder for run outputs.</t>
+          <t>Scaling on c(h, o_p) in selection criterion c_2.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>output_prefix</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>run</t>
-        </is>
+          <t>heuristic_wait_limit</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>9999</v>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>Prefix for run subfolder name.</t>
+          <t>Epsilon bound on total wait time.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
+          <t>apply_2opt</t>
+        </is>
+      </c>
+      <c r="B53" t="b">
+        <v>1</v>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>Run 2-opt local search after construction (lex-aware comparator).</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>apply_or_opt</t>
+        </is>
+      </c>
+      <c r="B54" t="b">
+        <v>1</v>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>Run Or-opt-on-pairs after 2-opt (lex-aware comparator).</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>solomon_backtrack_max_depth</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>20</v>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>Bounded-depth backtracking when greedy reaches infeasible_unrouted. 0 disables. n=20 instances need &gt;=15-17.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>solomon_multistart</t>
+        </is>
+      </c>
+      <c r="B56" t="b">
+        <v>1</v>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>When the requested bias fails after backtracking, retry under the other stock biases (route_duration → wait_time → balanced → extended).</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>solomon_random_restarts</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>20</v>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>After the 6 stock biases fail, try this many random alpha triples (log-uniform). 0 disables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>solomon_shuffle_restarts</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>100</v>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>After random alpha-restarts fail, try this many SHUFFLED-ORDER restarts: each picks a random insertion order over |P| parts. Defeats tight single-route instances. 0 disables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>solomon_random_seed</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>42</v>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>Seed for the random alpha-restarts AND shuffled-order restarts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t># VERIFICATION &amp; VISUALIZATION</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>auto_verify</t>
+        </is>
+      </c>
+      <c r="B61" t="b">
+        <v>1</v>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>Run verify.py on the solution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>verify_on_fail</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>raise</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>'raise' or 'warn' on verification failures.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>auto_visualize</t>
+        </is>
+      </c>
+      <c r="B63" t="b">
+        <v>1</v>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>Render Gantt / route / wait plots after each solve.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t># OUTPUT</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>output_dir</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>results</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>Destination folder for run outputs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>output_prefix</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>run</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>Prefix for run subfolder name.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
           <t>write_full_var_sheets</t>
         </is>
       </c>
-      <c r="B53" t="b">
-        <v>1</v>
-      </c>
-      <c r="C53" s="3" t="inlineStr">
+      <c r="B67" t="b">
+        <v>1</v>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
         <is>
           <t>Write per-variable sheets to result.xlsx (large files for big instances).</t>
         </is>

</xml_diff>